<commit_message>
User Access Maintenance FRS in BDOI's template v1.2: BDOI's FRS kept word for word, full BRD coverage in the mapping, items elaborated with acceptance criteria, new items FRUM.009-013, Annexes J-R with the observations for BDOI decision; review copy with the additions highlighted
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/Comparisons/BIBS_Comparison_BRD-11_BDOI_FRS_vs_BIBS_FRS_User_Access_Maintenance_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/Comparisons/BIBS_Comparison_BRD-11_BDOI_FRS_vs_BIBS_FRS_User_Access_Maintenance_v1.0.xlsx
@@ -1579,7 +1579,7 @@
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
-          <t>Keep BDOI's capabilities as the System Administrator's implementation of an approved group-profile request (FRUM.005.02 to .04, FRUM.006.04 to .06).</t>
+          <t>Keep BDOI's capabilities as the System Administrator's implementation of an approved group-profile request (FRUM.005.02 to .04, FRUM.006.04).</t>
         </is>
       </c>
       <c r="K7" s="12" t="inlineStr">
@@ -5085,7 +5085,7 @@
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>Under each item: our rules, validations, fields, statuses, approvals and messages as "The system shall ..." statements, then numbered acceptance criteria; new sub-items (FRUM.001.05, .06; FRUM.002.03; FRUM.003.04; FRUM.005.02-.06; FRUM.006.04-.06; FRUM.007.03; FRUM.008.04)</t>
+          <t>Under each item: our rules, validations, fields, statuses, approvals and messages as "The system shall ..." statements, then numbered acceptance criteria; new sub-items (FRUM.001.05, .06; FRUM.002.03; FRUM.003.04; FRUM.005.02-.06; FRUM.006.04; FRUM.007.03; FRUM.008.04)</t>
         </is>
       </c>
       <c r="D8" s="12" t="inlineStr">
@@ -20841,7 +20841,7 @@
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>New FRUM.005.02 to .04 and FRUM.006.04 to .06</t>
+          <t>New FRUM.005.02 to .04 and FRUM.006.04</t>
         </is>
       </c>
       <c r="D26" s="29" t="inlineStr">

</xml_diff>